<commit_message>
UpDate Automation n8n the DashBoard Streamit
</commit_message>
<xml_diff>
--- a/Projeto-custo-diário-solicitações-de-depósitos.xlsx
+++ b/Projeto-custo-diário-solicitações-de-depósitos.xlsx
@@ -472,7 +472,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" t="str">
         <v>81803</v>
       </c>
       <c r="B2" t="str">
@@ -496,7 +496,7 @@
       <c r="H2" t="str">
         <v xml:space="preserve">Marcio de Azevedo santos </v>
       </c>
-      <c r="I2">
+      <c r="I2" t="str">
         <v>350</v>
       </c>
       <c r="J2" t="str">
@@ -514,7 +514,7 @@
       <c r="N2" t="str">
         <v>252740</v>
       </c>
-      <c r="O2">
+      <c r="O2" t="str">
         <v>46028.78313657407</v>
       </c>
       <c r="P2" t="str">
@@ -523,7 +523,7 @@
       <c r="Q2" t="str">
         <v>32646446810</v>
       </c>
-      <c r="R2">
+      <c r="R2" t="str">
         <v>46028.82697916667</v>
       </c>
       <c r="S2" t="str">
@@ -531,7 +531,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="str">
         <v>81802</v>
       </c>
       <c r="B3" t="str">
@@ -555,7 +555,7 @@
       <c r="H3" t="str">
         <v>JOSENILDO FERREIRA CALADO</v>
       </c>
-      <c r="I3">
+      <c r="I3" t="str">
         <v>100</v>
       </c>
       <c r="J3" t="str">
@@ -573,7 +573,7 @@
       <c r="N3" t="str">
         <v>OS-252737</v>
       </c>
-      <c r="O3">
+      <c r="O3" t="str">
         <v>46028.78210648148</v>
       </c>
       <c r="P3" t="str">
@@ -582,7 +582,7 @@
       <c r="Q3" t="str">
         <v>CNPJ-16.852.O26/0001-06</v>
       </c>
-      <c r="R3">
+      <c r="R3" t="str">
         <v>46028.827048611114</v>
       </c>
       <c r="S3" t="str">
@@ -593,7 +593,7 @@
       </c>
     </row>
     <row r="4" xml:space="preserve">
-      <c r="A4">
+      <c r="A4" t="str">
         <v>81797</v>
       </c>
       <c r="B4" t="str">
@@ -621,7 +621,7 @@
       <c r="H4" t="str">
         <v>Marcelo Moura de Castro</v>
       </c>
-      <c r="I4">
+      <c r="I4" t="str">
         <v>75</v>
       </c>
       <c r="J4" t="str">
@@ -639,7 +639,7 @@
       <c r="N4" t="str">
         <v>252722</v>
       </c>
-      <c r="O4">
+      <c r="O4" t="str">
         <v>46028.73917824074</v>
       </c>
       <c r="P4" t="str">
@@ -648,7 +648,7 @@
       <c r="Q4" t="str">
         <v>CPF 27121916843</v>
       </c>
-      <c r="R4">
+      <c r="R4" t="str">
         <v>46028.826585648145</v>
       </c>
       <c r="S4" t="str">
@@ -662,7 +662,7 @@
       </c>
     </row>
     <row r="5" xml:space="preserve">
-      <c r="A5">
+      <c r="A5" t="str">
         <v>81795</v>
       </c>
       <c r="B5" t="str">
@@ -687,7 +687,7 @@
       <c r="G5" t="str">
         <v>Layza Nascimento Fagundes da Costa</v>
       </c>
-      <c r="I5">
+      <c r="I5" t="str">
         <v>2094</v>
       </c>
       <c r="J5" t="str">
@@ -705,7 +705,7 @@
       <c r="N5" t="str">
         <v>252718</v>
       </c>
-      <c r="O5">
+      <c r="O5" t="str">
         <v>46028.73599537037</v>
       </c>
       <c r="P5" t="str">
@@ -714,7 +714,7 @@
       <c r="Q5" t="str">
         <v xml:space="preserve"> 61529835000128 </v>
       </c>
-      <c r="R5">
+      <c r="R5" t="str">
         <v>46028.82662037037</v>
       </c>
       <c r="S5" t="str">
@@ -725,7 +725,7 @@
       </c>
     </row>
     <row r="6" xml:space="preserve">
-      <c r="A6">
+      <c r="A6" t="str">
         <v>81790</v>
       </c>
       <c r="B6" t="str">
@@ -750,7 +750,7 @@
       <c r="G6" t="str">
         <v>Layza Nascimento Fagundes da Costa</v>
       </c>
-      <c r="I6">
+      <c r="I6" t="str">
         <v>300</v>
       </c>
       <c r="J6" t="str">
@@ -768,7 +768,7 @@
       <c r="N6" t="str">
         <v>252696</v>
       </c>
-      <c r="O6">
+      <c r="O6" t="str">
         <v>46028.727326388886</v>
       </c>
       <c r="P6" t="str">
@@ -777,7 +777,7 @@
       <c r="Q6" t="str">
         <v>CNPJ 36.649.112/0001-15</v>
       </c>
-      <c r="R6">
+      <c r="R6" t="str">
         <v>46028.7690625</v>
       </c>
       <c r="S6" t="str">
@@ -785,7 +785,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
+      <c r="A7" t="str">
         <v>81785</v>
       </c>
       <c r="B7" t="str">
@@ -809,7 +809,7 @@
       <c r="H7" t="str">
         <v>Vanilson Monteiro Lopes</v>
       </c>
-      <c r="I7">
+      <c r="I7" t="str">
         <v>120</v>
       </c>
       <c r="J7" t="str">
@@ -827,7 +827,7 @@
       <c r="N7" t="str">
         <v>252677</v>
       </c>
-      <c r="O7">
+      <c r="O7" t="str">
         <v>46028.70190972222</v>
       </c>
       <c r="P7" t="str">
@@ -836,7 +836,7 @@
       <c r="Q7" t="str">
         <v>CNPJ 13665260000128</v>
       </c>
-      <c r="R7">
+      <c r="R7" t="str">
         <v>46028.768275462964</v>
       </c>
       <c r="S7" t="str">
@@ -847,7 +847,7 @@
       </c>
     </row>
     <row r="8" xml:space="preserve">
-      <c r="A8">
+      <c r="A8" t="str">
         <v>81776</v>
       </c>
       <c r="B8" t="str">
@@ -871,7 +871,7 @@
       <c r="G8" t="str">
         <v>Layza Nascimento Fagundes da Costa</v>
       </c>
-      <c r="I8">
+      <c r="I8" t="str">
         <v>300</v>
       </c>
       <c r="K8" t="str">
@@ -886,7 +886,7 @@
       <c r="N8" t="str">
         <v>252646</v>
       </c>
-      <c r="O8">
+      <c r="O8" t="str">
         <v>46028.64429398148</v>
       </c>
       <c r="P8" t="str">
@@ -895,7 +895,7 @@
       <c r="Q8" t="str">
         <v>CNPJ: 44879973000118</v>
       </c>
-      <c r="R8">
+      <c r="R8" t="str">
         <v>46028.768171296295</v>
       </c>
       <c r="S8" t="str">
@@ -906,7 +906,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
+      <c r="A9" t="str">
         <v>81774</v>
       </c>
       <c r="B9" t="str">
@@ -930,7 +930,7 @@
       <c r="H9" t="str">
         <v>RENATO CAFUNDO</v>
       </c>
-      <c r="I9">
+      <c r="I9" t="str">
         <v>500</v>
       </c>
       <c r="J9" t="str">
@@ -948,7 +948,7 @@
       <c r="N9" t="str">
         <v>OS-252537</v>
       </c>
-      <c r="O9">
+      <c r="O9" t="str">
         <v>46028.63644675926</v>
       </c>
       <c r="P9" t="str">
@@ -957,7 +957,7 @@
       <c r="Q9" t="str">
         <v xml:space="preserve">CNPJ-55.632.796/0001-97 </v>
       </c>
-      <c r="R9">
+      <c r="R9" t="str">
         <v>46028.66987268518</v>
       </c>
       <c r="S9" t="str">
@@ -968,7 +968,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
+      <c r="A10" t="str">
         <v>81773</v>
       </c>
       <c r="B10" t="str">
@@ -992,7 +992,7 @@
       <c r="H10" t="str">
         <v xml:space="preserve">MARCIO ROGERIO CASTANHO </v>
       </c>
-      <c r="I10">
+      <c r="I10" t="str">
         <v>60</v>
       </c>
       <c r="J10" t="str">
@@ -1010,7 +1010,7 @@
       <c r="N10" t="str">
         <v>OS-252644</v>
       </c>
-      <c r="O10">
+      <c r="O10" t="str">
         <v>46028.631516203706</v>
       </c>
       <c r="P10" t="str">
@@ -1019,7 +1019,7 @@
       <c r="Q10" t="str">
         <v>CPF-838.952.481-34</v>
       </c>
-      <c r="R10">
+      <c r="R10" t="str">
         <v>46028.66144675926</v>
       </c>
       <c r="S10" t="str">
@@ -1030,7 +1030,7 @@
       </c>
     </row>
     <row r="11" xml:space="preserve">
-      <c r="A11">
+      <c r="A11" t="str">
         <v>81772</v>
       </c>
       <c r="B11" t="str">
@@ -1058,7 +1058,7 @@
       <c r="H11" t="str">
         <v>Douglas Gomes Ishibashi</v>
       </c>
-      <c r="I11">
+      <c r="I11" t="str">
         <v>50</v>
       </c>
       <c r="J11" t="str">
@@ -1076,7 +1076,7 @@
       <c r="N11" t="str">
         <v>252645</v>
       </c>
-      <c r="O11">
+      <c r="O11" t="str">
         <v>46028.63141203704</v>
       </c>
       <c r="P11" t="str">
@@ -1085,7 +1085,7 @@
       <c r="Q11" t="str">
         <v xml:space="preserve">068.705.666-74 </v>
       </c>
-      <c r="R11">
+      <c r="R11" t="str">
         <v>46028.76758101852</v>
       </c>
       <c r="S11" t="str">
@@ -1096,7 +1096,7 @@
       </c>
     </row>
     <row r="12" xml:space="preserve">
-      <c r="A12">
+      <c r="A12" t="str">
         <v>81746</v>
       </c>
       <c r="B12" t="str">
@@ -1121,7 +1121,7 @@
       <c r="G12" t="str">
         <v>Layza Nascimento Fagundes da Costa</v>
       </c>
-      <c r="I12">
+      <c r="I12" t="str">
         <v>80</v>
       </c>
       <c r="K12" t="str">
@@ -1136,13 +1136,13 @@
       <c r="N12" t="str">
         <v>1523</v>
       </c>
-      <c r="O12">
+      <c r="O12" t="str">
         <v>46028.52547453704</v>
       </c>
       <c r="P12" t="str">
         <v xml:space="preserve">Thales André Gomes de Sá </v>
       </c>
-      <c r="R12">
+      <c r="R12" t="str">
         <v>46028.61241898148</v>
       </c>
       <c r="S12" t="str">
@@ -1153,7 +1153,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
+      <c r="A13" t="str">
         <v>81745</v>
       </c>
       <c r="B13" t="str">
@@ -1174,7 +1174,7 @@
       <c r="G13" t="str">
         <v>Mickaelly Soares de  Siqueira</v>
       </c>
-      <c r="I13">
+      <c r="I13" t="str">
         <v>2432</v>
       </c>
       <c r="J13" t="str">
@@ -1192,7 +1192,7 @@
       <c r="N13" t="str">
         <v>252560</v>
       </c>
-      <c r="O13">
+      <c r="O13" t="str">
         <v>46028.52310185185</v>
       </c>
       <c r="P13" t="str">
@@ -1201,7 +1201,7 @@
       <c r="Q13" t="str">
         <v>26.345.971/0001-67</v>
       </c>
-      <c r="R13">
+      <c r="R13" t="str">
         <v>46028.61237268519</v>
       </c>
       <c r="S13" t="str">
@@ -1209,7 +1209,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
+      <c r="A14" t="str">
         <v>81744</v>
       </c>
       <c r="B14" t="str">
@@ -1230,7 +1230,7 @@
       <c r="G14" t="str">
         <v>Mickaelly Soares de  Siqueira</v>
       </c>
-      <c r="I14">
+      <c r="I14" t="str">
         <v>243200</v>
       </c>
       <c r="J14" t="str">
@@ -1248,7 +1248,7 @@
       <c r="N14" t="str">
         <v>252560</v>
       </c>
-      <c r="O14">
+      <c r="O14" t="str">
         <v>46028.51954861111</v>
       </c>
       <c r="P14" t="str">
@@ -1257,7 +1257,7 @@
       <c r="Q14" t="str">
         <v>26.345.971/0001-67</v>
       </c>
-      <c r="R14">
+      <c r="R14" t="str">
         <v>46028.52075231481</v>
       </c>
       <c r="S14" t="str">
@@ -1265,7 +1265,7 @@
       </c>
     </row>
     <row r="15" xml:space="preserve">
-      <c r="A15">
+      <c r="A15" t="str">
         <v>81742</v>
       </c>
       <c r="B15" t="str">
@@ -1293,7 +1293,7 @@
       <c r="H15" t="str">
         <v>EDUARDO HENRIQUE AGUIAR DE PAIVA</v>
       </c>
-      <c r="I15">
+      <c r="I15" t="str">
         <v>200</v>
       </c>
       <c r="J15" t="str">
@@ -1311,7 +1311,7 @@
       <c r="N15" t="str">
         <v>252547 / 252550</v>
       </c>
-      <c r="O15">
+      <c r="O15" t="str">
         <v>46028.514502314814</v>
       </c>
       <c r="P15" t="str">
@@ -1320,7 +1320,7 @@
       <c r="Q15" t="str">
         <v>925.538.261-68</v>
       </c>
-      <c r="R15">
+      <c r="R15" t="str">
         <v>46028.66978009259</v>
       </c>
       <c r="S15" t="str">
@@ -1340,7 +1340,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
+      <c r="A16" t="str">
         <v>81741</v>
       </c>
       <c r="B16" t="str">
@@ -1361,7 +1361,7 @@
       <c r="G16" t="str">
         <v>Mickaelly Soares de  Siqueira</v>
       </c>
-      <c r="I16">
+      <c r="I16" t="str">
         <v>45</v>
       </c>
       <c r="J16" t="str">
@@ -1379,7 +1379,7 @@
       <c r="N16" t="str">
         <v>252551</v>
       </c>
-      <c r="O16">
+      <c r="O16" t="str">
         <v>46028.508043981485</v>
       </c>
       <c r="P16" t="str">
@@ -1388,7 +1388,7 @@
       <c r="Q16" t="str">
         <v>19 98188 1225</v>
       </c>
-      <c r="R16">
+      <c r="R16" t="str">
         <v>46028.61216435185</v>
       </c>
       <c r="S16" t="str">
@@ -1396,7 +1396,7 @@
       </c>
     </row>
     <row r="17" xml:space="preserve">
-      <c r="A17">
+      <c r="A17" t="str">
         <v>81738</v>
       </c>
       <c r="B17" t="str">
@@ -1423,7 +1423,7 @@
       <c r="H17" t="str">
         <v>ANGEL ANTONIO FUENMAYOR SEMPRUN</v>
       </c>
-      <c r="I17">
+      <c r="I17" t="str">
         <v>120</v>
       </c>
       <c r="J17" t="str">
@@ -1441,7 +1441,7 @@
       <c r="N17" t="str">
         <v>252531</v>
       </c>
-      <c r="O17">
+      <c r="O17" t="str">
         <v>46028.50071759259</v>
       </c>
       <c r="P17" t="str">
@@ -1450,7 +1450,7 @@
       <c r="Q17" t="str">
         <v>712.558.811-51</v>
       </c>
-      <c r="R17">
+      <c r="R17" t="str">
         <v>46028.66957175926</v>
       </c>
       <c r="S17" t="str">
@@ -1470,7 +1470,7 @@
       </c>
     </row>
     <row r="18" xml:space="preserve">
-      <c r="A18">
+      <c r="A18" t="str">
         <v>81737</v>
       </c>
       <c r="B18" t="str">
@@ -1496,7 +1496,7 @@
       <c r="H18" t="str">
         <v xml:space="preserve"> Roberto José da Silva</v>
       </c>
-      <c r="I18">
+      <c r="I18" t="str">
         <v>110</v>
       </c>
       <c r="J18" t="str">
@@ -1514,10 +1514,10 @@
       <c r="N18" t="str">
         <v>252512</v>
       </c>
-      <c r="O18">
+      <c r="O18" t="str">
         <v>46028.488287037035</v>
       </c>
-      <c r="R18">
+      <c r="R18" t="str">
         <v>46028.61153935185</v>
       </c>
       <c r="S18" t="str">
@@ -1528,7 +1528,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
+      <c r="A19" t="str">
         <v>81722</v>
       </c>
       <c r="B19" t="str">
@@ -1552,7 +1552,7 @@
       <c r="H19" t="str">
         <v>IGOR GABRIEL PONTES LEONARDO</v>
       </c>
-      <c r="I19">
+      <c r="I19" t="str">
         <v>420</v>
       </c>
       <c r="J19" t="str">
@@ -1570,7 +1570,7 @@
       <c r="N19" t="str">
         <v>OS-252471</v>
       </c>
-      <c r="O19">
+      <c r="O19" t="str">
         <v>46028.44850694444</v>
       </c>
       <c r="P19" t="str">
@@ -1579,7 +1579,7 @@
       <c r="Q19" t="str">
         <v xml:space="preserve">CNPJ-10.318.150/0001-00 </v>
       </c>
-      <c r="R19">
+      <c r="R19" t="str">
         <v>46028.51329861111</v>
       </c>
       <c r="S19" t="str">
@@ -1590,7 +1590,7 @@
       </c>
     </row>
     <row r="20" xml:space="preserve">
-      <c r="A20">
+      <c r="A20" t="str">
         <v>81719</v>
       </c>
       <c r="B20" t="str">
@@ -1616,7 +1616,7 @@
       <c r="H20" t="str">
         <v>Joelson Souza de Oliveira</v>
       </c>
-      <c r="I20">
+      <c r="I20" t="str">
         <v>100</v>
       </c>
       <c r="J20" t="str">
@@ -1634,13 +1634,13 @@
       <c r="N20" t="str">
         <v>252480</v>
       </c>
-      <c r="O20">
+      <c r="O20" t="str">
         <v>46028.442777777775</v>
       </c>
       <c r="P20" t="str">
         <v>Auto elétrica iturama</v>
       </c>
-      <c r="R20">
+      <c r="R20" t="str">
         <v>46028.46449074074</v>
       </c>
       <c r="S20" t="str">
@@ -1651,7 +1651,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21">
+      <c r="A21" t="str">
         <v>81710</v>
       </c>
       <c r="B21" t="str">
@@ -1672,7 +1672,7 @@
       <c r="G21" t="str">
         <v>Mickaelly Soares de  Siqueira</v>
       </c>
-      <c r="I21">
+      <c r="I21" t="str">
         <v>93</v>
       </c>
       <c r="J21" t="str">
@@ -1690,7 +1690,7 @@
       <c r="N21" t="str">
         <v>252418</v>
       </c>
-      <c r="O21">
+      <c r="O21" t="str">
         <v>46028.40456018518</v>
       </c>
       <c r="P21" t="str">
@@ -1699,7 +1699,7 @@
       <c r="Q21" t="str">
         <v>50497778000126</v>
       </c>
-      <c r="R21">
+      <c r="R21" t="str">
         <v>46028.463842592595</v>
       </c>
       <c r="S21" t="str">
@@ -1707,7 +1707,7 @@
       </c>
     </row>
     <row r="22" xml:space="preserve">
-      <c r="A22">
+      <c r="A22" t="str">
         <v>81696</v>
       </c>
       <c r="B22" t="str">
@@ -1733,7 +1733,7 @@
       <c r="H22" t="str">
         <v xml:space="preserve">Claudio Antonio dos Anjos Nunes </v>
       </c>
-      <c r="I22">
+      <c r="I22" t="str">
         <v>150</v>
       </c>
       <c r="J22" t="str">
@@ -1751,10 +1751,10 @@
       <c r="N22" t="str">
         <v>252365</v>
       </c>
-      <c r="O22">
+      <c r="O22" t="str">
         <v>46028.35649305556</v>
       </c>
-      <c r="R22">
+      <c r="R22" t="str">
         <v>46028.370520833334</v>
       </c>
       <c r="S22" t="str">
@@ -1765,7 +1765,7 @@
       </c>
     </row>
     <row r="23" xml:space="preserve">
-      <c r="A23">
+      <c r="A23" t="str">
         <v>81695</v>
       </c>
       <c r="B23" t="str">
@@ -1792,7 +1792,7 @@
       <c r="H23" t="str">
         <v>-</v>
       </c>
-      <c r="I23">
+      <c r="I23" t="str">
         <v>200</v>
       </c>
       <c r="J23" t="str">
@@ -1810,7 +1810,7 @@
       <c r="N23" t="str">
         <v>252353</v>
       </c>
-      <c r="O23">
+      <c r="O23" t="str">
         <v>46028.35377314815</v>
       </c>
       <c r="P23" t="str">
@@ -1819,7 +1819,7 @@
       <c r="Q23" t="str">
         <v>387.385.678.65</v>
       </c>
-      <c r="R23">
+      <c r="R23" t="str">
         <v>46028.40372685185</v>
       </c>
       <c r="S23" t="str">
@@ -1839,7 +1839,7 @@
       </c>
     </row>
     <row r="24" xml:space="preserve">
-      <c r="A24">
+      <c r="A24" t="str">
         <v>81694</v>
       </c>
       <c r="B24" t="str">
@@ -1865,7 +1865,7 @@
       <c r="H24" t="str">
         <v>Manoel Boanerges da rocha Ferraz neto</v>
       </c>
-      <c r="I24">
+      <c r="I24" t="str">
         <v>400</v>
       </c>
       <c r="J24" t="str">
@@ -1883,13 +1883,13 @@
       <c r="N24" t="str">
         <v>252348</v>
       </c>
-      <c r="O24">
+      <c r="O24" t="str">
         <v>46028.34918981481</v>
       </c>
       <c r="P24" t="str">
         <v>Eliak joseph da silva</v>
       </c>
-      <c r="R24">
+      <c r="R24" t="str">
         <v>46028.404594907406</v>
       </c>
       <c r="S24" t="str">
@@ -1900,7 +1900,7 @@
       </c>
     </row>
     <row r="25" xml:space="preserve">
-      <c r="A25">
+      <c r="A25" t="str">
         <v>81693</v>
       </c>
       <c r="B25" t="str">
@@ -1926,7 +1926,7 @@
       <c r="H25" t="str">
         <v>Valdomiro Sabino</v>
       </c>
-      <c r="I25">
+      <c r="I25" t="str">
         <v>890</v>
       </c>
       <c r="J25" t="str">
@@ -1944,13 +1944,13 @@
       <c r="N25" t="str">
         <v>252320</v>
       </c>
-      <c r="O25">
+      <c r="O25" t="str">
         <v>46028.33273148148</v>
       </c>
       <c r="P25" t="str">
         <v>BRUNO BELOTO PIZOL</v>
       </c>
-      <c r="R25">
+      <c r="R25" t="str">
         <v>46028.40362268518</v>
       </c>
       <c r="S25" t="str">
@@ -1961,7 +1961,7 @@
       </c>
     </row>
     <row r="26" xml:space="preserve">
-      <c r="A26">
+      <c r="A26" t="str">
         <v>81691</v>
       </c>
       <c r="B26" t="str">
@@ -1987,7 +1987,7 @@
       <c r="H26" t="str">
         <v>Valdomiro Sabino</v>
       </c>
-      <c r="I26">
+      <c r="I26" t="str">
         <v>380</v>
       </c>
       <c r="J26" t="str">
@@ -2005,13 +2005,13 @@
       <c r="N26" t="str">
         <v>252283</v>
       </c>
-      <c r="O26">
+      <c r="O26" t="str">
         <v>46028.299780092595</v>
       </c>
       <c r="P26" t="str">
         <v>BRUNO BELOTO PIZOL</v>
       </c>
-      <c r="R26">
+      <c r="R26" t="str">
         <v>46028.37037037037</v>
       </c>
       <c r="S26" t="str">
@@ -2022,7 +2022,7 @@
       </c>
     </row>
     <row r="27" xml:space="preserve">
-      <c r="A27">
+      <c r="A27" t="str">
         <v>81690</v>
       </c>
       <c r="B27" t="str">
@@ -2048,7 +2048,7 @@
       <c r="H27" t="str">
         <v>BRUNO GUILHERME VENTURA CONSTANTE</v>
       </c>
-      <c r="I27">
+      <c r="I27" t="str">
         <v>600</v>
       </c>
       <c r="J27" t="str">
@@ -2066,13 +2066,13 @@
       <c r="N27" t="str">
         <v>252277</v>
       </c>
-      <c r="O27">
+      <c r="O27" t="str">
         <v>46028.28462962963</v>
       </c>
       <c r="P27" t="str">
         <v>MAYKO WM DOS SANTOS SERVIÇOS DE SOLDAS ESPECIAIS</v>
       </c>
-      <c r="R27">
+      <c r="R27" t="str">
         <v>46028.36988425926</v>
       </c>
       <c r="S27" t="str">
@@ -2083,7 +2083,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28">
+      <c r="A28" t="str">
         <v>81689</v>
       </c>
       <c r="B28" t="str">
@@ -2107,7 +2107,7 @@
       <c r="H28" t="str">
         <v xml:space="preserve">SAULO SATHLER DUARTE </v>
       </c>
-      <c r="I28">
+      <c r="I28" t="str">
         <v>490</v>
       </c>
       <c r="J28" t="str">
@@ -2122,13 +2122,13 @@
       <c r="M28" t="str">
         <v>Membros de Caixa Km 18</v>
       </c>
-      <c r="O28">
+      <c r="O28" t="str">
         <v>46028.24657407407</v>
       </c>
       <c r="P28" t="str">
         <v xml:space="preserve">SAULO SATHLER DUARTE </v>
       </c>
-      <c r="R28">
+      <c r="R28" t="str">
         <v>46028.403078703705</v>
       </c>
       <c r="S28" t="str">
@@ -2136,7 +2136,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29">
+      <c r="A29" t="str">
         <v>81677</v>
       </c>
       <c r="B29" t="str">
@@ -2160,7 +2160,7 @@
       <c r="H29" t="str">
         <v>VALTER SANTOS SANTANA</v>
       </c>
-      <c r="I29">
+      <c r="I29" t="str">
         <v>90</v>
       </c>
       <c r="J29" t="str">
@@ -2178,7 +2178,7 @@
       <c r="N29" t="str">
         <v>OS-252246</v>
       </c>
-      <c r="O29">
+      <c r="O29" t="str">
         <v>46027.767488425925</v>
       </c>
       <c r="P29" t="str">
@@ -2187,7 +2187,7 @@
       <c r="Q29" t="str">
         <v>CPF-292.260.578-77</v>
       </c>
-      <c r="R29">
+      <c r="R29" t="str">
         <v>46027.85046296296</v>
       </c>
       <c r="S29" t="str">
@@ -2198,7 +2198,7 @@
       </c>
     </row>
     <row r="30" xml:space="preserve">
-      <c r="A30">
+      <c r="A30" t="str">
         <v>81663</v>
       </c>
       <c r="B30" t="str">
@@ -2226,7 +2226,7 @@
       <c r="H30" t="str">
         <v xml:space="preserve">Lucas Araújo Souza </v>
       </c>
-      <c r="I30">
+      <c r="I30" t="str">
         <v>80</v>
       </c>
       <c r="J30" t="str">
@@ -2244,7 +2244,7 @@
       <c r="N30" t="str">
         <v>252219</v>
       </c>
-      <c r="O30">
+      <c r="O30" t="str">
         <v>46027.733622685184</v>
       </c>
       <c r="P30" t="str">
@@ -2253,7 +2253,7 @@
       <c r="Q30" t="str">
         <v>052.494.311-78</v>
       </c>
-      <c r="R30">
+      <c r="R30" t="str">
         <v>46027.75193287037</v>
       </c>
       <c r="S30" t="str">
@@ -2264,7 +2264,7 @@
       </c>
     </row>
     <row r="31" xml:space="preserve">
-      <c r="A31">
+      <c r="A31" t="str">
         <v>81662</v>
       </c>
       <c r="B31" t="str">
@@ -2290,7 +2290,7 @@
       <c r="H31" t="str">
         <v>Carlos Antônio da silva</v>
       </c>
-      <c r="I31">
+      <c r="I31" t="str">
         <v>80</v>
       </c>
       <c r="K31" t="str">
@@ -2305,7 +2305,7 @@
       <c r="N31" t="str">
         <v>O.S: 252201</v>
       </c>
-      <c r="O31">
+      <c r="O31" t="str">
         <v>46027.72221064815</v>
       </c>
       <c r="P31" t="str">
@@ -2314,7 +2314,7 @@
       <c r="Q31" t="str">
         <v>CPF 11222268884</v>
       </c>
-      <c r="R31">
+      <c r="R31" t="str">
         <v>46027.75188657407</v>
       </c>
       <c r="S31" t="str">
@@ -2334,7 +2334,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32">
+      <c r="A32" t="str">
         <v>81655</v>
       </c>
       <c r="B32" t="str">
@@ -2358,7 +2358,7 @@
       <c r="H32" t="str">
         <v>VALTER SANTOS SANTANA</v>
       </c>
-      <c r="I32">
+      <c r="I32" t="str">
         <v>85</v>
       </c>
       <c r="J32" t="str">
@@ -2376,7 +2376,7 @@
       <c r="N32" t="str">
         <v>OS-252170</v>
       </c>
-      <c r="O32">
+      <c r="O32" t="str">
         <v>46027.69436342592</v>
       </c>
       <c r="P32" t="str">
@@ -2385,7 +2385,7 @@
       <c r="Q32" t="str">
         <v>CPF-292.260.578-77</v>
       </c>
-      <c r="R32">
+      <c r="R32" t="str">
         <v>46027.720729166664</v>
       </c>
       <c r="S32" t="str">
@@ -2396,7 +2396,7 @@
       </c>
     </row>
     <row r="33" xml:space="preserve">
-      <c r="A33">
+      <c r="A33" t="str">
         <v>81652</v>
       </c>
       <c r="B33" t="str">
@@ -2423,7 +2423,7 @@
       <c r="H33" t="str">
         <v>Gladson soares Rodrigues</v>
       </c>
-      <c r="I33">
+      <c r="I33" t="str">
         <v>120</v>
       </c>
       <c r="J33" t="str">
@@ -2441,7 +2441,7 @@
       <c r="N33" t="str">
         <v>252151</v>
       </c>
-      <c r="O33">
+      <c r="O33" t="str">
         <v>46027.684432870374</v>
       </c>
       <c r="P33" t="str">
@@ -2450,7 +2450,7 @@
       <c r="Q33" t="str">
         <v xml:space="preserve"> 58257063649</v>
       </c>
-      <c r="R33">
+      <c r="R33" t="str">
         <v>46027.72048611111</v>
       </c>
       <c r="S33" t="str">
@@ -2464,7 +2464,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34">
+      <c r="A34" t="str">
         <v>81651</v>
       </c>
       <c r="B34" t="str">
@@ -2488,7 +2488,7 @@
       <c r="H34" t="str">
         <v xml:space="preserve"> Severino Alberto de Freitas</v>
       </c>
-      <c r="I34">
+      <c r="I34" t="str">
         <v>150</v>
       </c>
       <c r="J34" t="str">
@@ -2506,7 +2506,7 @@
       <c r="N34" t="str">
         <v>252146</v>
       </c>
-      <c r="O34">
+      <c r="O34" t="str">
         <v>46027.67870370371</v>
       </c>
       <c r="P34" t="str">
@@ -2515,7 +2515,7 @@
       <c r="Q34" t="str">
         <v>CPF 02822727473</v>
       </c>
-      <c r="R34">
+      <c r="R34" t="str">
         <v>46027.720405092594</v>
       </c>
       <c r="S34" t="str">
@@ -2526,7 +2526,7 @@
       </c>
     </row>
     <row r="35" xml:space="preserve">
-      <c r="A35">
+      <c r="A35" t="str">
         <v>81646</v>
       </c>
       <c r="B35" t="str">
@@ -2548,7 +2548,7 @@
       <c r="G35" t="str">
         <v>Bruna Vieira da Silva</v>
       </c>
-      <c r="I35">
+      <c r="I35" t="str">
         <v>600</v>
       </c>
       <c r="J35" t="str">
@@ -2566,7 +2566,7 @@
       <c r="N35" t="str">
         <v>252131</v>
       </c>
-      <c r="O35">
+      <c r="O35" t="str">
         <v>46027.66509259259</v>
       </c>
       <c r="P35" t="str">
@@ -2575,7 +2575,7 @@
       <c r="Q35" t="str">
         <v>14611199878</v>
       </c>
-      <c r="R35">
+      <c r="R35" t="str">
         <v>46027.72033564815</v>
       </c>
       <c r="S35" t="str">
@@ -2583,7 +2583,7 @@
       </c>
     </row>
     <row r="36" xml:space="preserve">
-      <c r="A36">
+      <c r="A36" t="str">
         <v>81645</v>
       </c>
       <c r="B36" t="str">
@@ -2608,7 +2608,7 @@
       <c r="G36" t="str">
         <v>Layza Nascimento Fagundes da Costa</v>
       </c>
-      <c r="I36">
+      <c r="I36" t="str">
         <v>400</v>
       </c>
       <c r="J36" t="str">
@@ -2626,7 +2626,7 @@
       <c r="N36" t="str">
         <v>252129</v>
       </c>
-      <c r="O36">
+      <c r="O36" t="str">
         <v>46027.66427083333</v>
       </c>
       <c r="P36" t="str">
@@ -2635,7 +2635,7 @@
       <c r="Q36" t="str">
         <v>71986338530</v>
       </c>
-      <c r="R36">
+      <c r="R36" t="str">
         <v>46027.720347222225</v>
       </c>
       <c r="S36" t="str">
@@ -2646,7 +2646,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37">
+      <c r="A37" t="str">
         <v>81643</v>
       </c>
       <c r="B37" t="str">
@@ -2670,7 +2670,7 @@
       <c r="H37" t="str">
         <v>Leopoldo Zimmermann</v>
       </c>
-      <c r="I37">
+      <c r="I37" t="str">
         <v>260</v>
       </c>
       <c r="J37" t="str">
@@ -2688,7 +2688,7 @@
       <c r="N37" t="str">
         <v>252111</v>
       </c>
-      <c r="O37">
+      <c r="O37" t="str">
         <v>46027.64606481481</v>
       </c>
       <c r="P37" t="str">
@@ -2697,7 +2697,7 @@
       <c r="Q37" t="str">
         <v>CPF 16170959827</v>
       </c>
-      <c r="R37">
+      <c r="R37" t="str">
         <v>46027.68311342593</v>
       </c>
       <c r="S37" t="str">
@@ -2708,7 +2708,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38">
+      <c r="A38" t="str">
         <v>81642</v>
       </c>
       <c r="B38" t="str">
@@ -2732,7 +2732,7 @@
       <c r="H38" t="str">
         <v>ROGERIO ASSIS LEÃO</v>
       </c>
-      <c r="I38">
+      <c r="I38" t="str">
         <v>195</v>
       </c>
       <c r="J38" t="str">
@@ -2750,7 +2750,7 @@
       <c r="N38" t="str">
         <v>OS-252104</v>
       </c>
-      <c r="O38">
+      <c r="O38" t="str">
         <v>46027.63700231481</v>
       </c>
       <c r="P38" t="str">
@@ -2759,7 +2759,7 @@
       <c r="Q38" t="str">
         <v>CPF-078.552.017-18</v>
       </c>
-      <c r="R38">
+      <c r="R38" t="str">
         <v>46027.68305555556</v>
       </c>
       <c r="S38" t="str">
@@ -2770,7 +2770,7 @@
       </c>
     </row>
     <row r="39" xml:space="preserve">
-      <c r="A39">
+      <c r="A39" t="str">
         <v>81641</v>
       </c>
       <c r="B39" t="str">
@@ -2798,7 +2798,7 @@
       <c r="H39" t="str">
         <v>-</v>
       </c>
-      <c r="I39">
+      <c r="I39" t="str">
         <v>2600</v>
       </c>
       <c r="J39" t="str">
@@ -2816,13 +2816,13 @@
       <c r="N39" t="str">
         <v>252101</v>
       </c>
-      <c r="O39">
+      <c r="O39" t="str">
         <v>46027.63653935185</v>
       </c>
       <c r="P39" t="str">
         <v>Carlos Alberto da Silva Vieira</v>
       </c>
-      <c r="R39">
+      <c r="R39" t="str">
         <v>46027.68299768519</v>
       </c>
       <c r="S39" t="str">
@@ -2842,7 +2842,7 @@
       </c>
     </row>
     <row r="40" xml:space="preserve">
-      <c r="A40">
+      <c r="A40" t="str">
         <v>81640</v>
       </c>
       <c r="B40" t="str">
@@ -2867,7 +2867,7 @@
       <c r="H40" t="str">
         <v>Carlos Eduardo macedo</v>
       </c>
-      <c r="I40">
+      <c r="I40" t="str">
         <v>500</v>
       </c>
       <c r="J40" t="str">
@@ -2885,7 +2885,7 @@
       <c r="N40" t="str">
         <v>252103</v>
       </c>
-      <c r="O40">
+      <c r="O40" t="str">
         <v>46027.63451388889</v>
       </c>
       <c r="P40" t="str">
@@ -2894,7 +2894,7 @@
       <c r="Q40" t="str">
         <v>CNPJ: 03.125.278/0001-83</v>
       </c>
-      <c r="R40">
+      <c r="R40" t="str">
         <v>46027.682604166665</v>
       </c>
       <c r="S40" t="str">
@@ -2905,7 +2905,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41">
+      <c r="A41" t="str">
         <v>81638</v>
       </c>
       <c r="B41" t="str">
@@ -2929,7 +2929,7 @@
       <c r="H41" t="str">
         <v>PATTERSON CARDOSO DOS SANTOS</v>
       </c>
-      <c r="I41">
+      <c r="I41" t="str">
         <v>50</v>
       </c>
       <c r="J41" t="str">
@@ -2947,7 +2947,7 @@
       <c r="N41" t="str">
         <v>OS-252100</v>
       </c>
-      <c r="O41">
+      <c r="O41" t="str">
         <v>46027.626388888886</v>
       </c>
       <c r="P41" t="str">
@@ -2956,7 +2956,7 @@
       <c r="Q41" t="str">
         <v>CPF-300.445.818-74</v>
       </c>
-      <c r="R41">
+      <c r="R41" t="str">
         <v>46027.65188657407</v>
       </c>
       <c r="S41" t="str">
@@ -2967,7 +2967,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42">
+      <c r="A42" t="str">
         <v>81635</v>
       </c>
       <c r="B42" t="str">
@@ -2988,7 +2988,7 @@
       <c r="G42" t="str">
         <v>Michele Brito da Silva</v>
       </c>
-      <c r="I42">
+      <c r="I42" t="str">
         <v>600</v>
       </c>
       <c r="J42" t="str">
@@ -3003,13 +3003,13 @@
       <c r="M42" t="str">
         <v>Membros de Caixa Km 18</v>
       </c>
-      <c r="O42">
+      <c r="O42" t="str">
         <v>46027.60230324074</v>
       </c>
       <c r="Q42" t="str">
         <v>14611199878</v>
       </c>
-      <c r="R42">
+      <c r="R42" t="str">
         <v>46027.63829861111</v>
       </c>
       <c r="S42" t="str">
@@ -3017,7 +3017,7 @@
       </c>
     </row>
     <row r="43" xml:space="preserve">
-      <c r="A43">
+      <c r="A43" t="str">
         <v>81634</v>
       </c>
       <c r="B43" t="str">
@@ -3044,7 +3044,7 @@
       <c r="H43" t="str">
         <v>Robertson Ulisses Ferreira</v>
       </c>
-      <c r="I43">
+      <c r="I43" t="str">
         <v>70</v>
       </c>
       <c r="J43" t="str">
@@ -3062,7 +3062,7 @@
       <c r="N43" t="str">
         <v>252084</v>
       </c>
-      <c r="O43">
+      <c r="O43" t="str">
         <v>46027.59446759259</v>
       </c>
       <c r="P43" t="str">
@@ -3071,7 +3071,7 @@
       <c r="Q43" t="str">
         <v>308.927.468-07</v>
       </c>
-      <c r="R43">
+      <c r="R43" t="str">
         <v>46027.6518287037</v>
       </c>
       <c r="S43" t="str">
@@ -3082,7 +3082,7 @@
       </c>
     </row>
     <row r="44" xml:space="preserve">
-      <c r="A44">
+      <c r="A44" t="str">
         <v>81633</v>
       </c>
       <c r="B44" t="str">
@@ -3110,7 +3110,7 @@
       <c r="H44" t="str">
         <v xml:space="preserve">Dione rosa madureira </v>
       </c>
-      <c r="I44">
+      <c r="I44" t="str">
         <v>80</v>
       </c>
       <c r="J44" t="str">
@@ -3128,7 +3128,7 @@
       <c r="N44" t="str">
         <v>252081</v>
       </c>
-      <c r="O44">
+      <c r="O44" t="str">
         <v>46027.58859953703</v>
       </c>
       <c r="P44" t="str">
@@ -3137,7 +3137,7 @@
       <c r="Q44" t="str">
         <v>CPF 09562399605</v>
       </c>
-      <c r="R44">
+      <c r="R44" t="str">
         <v>46027.61414351852</v>
       </c>
       <c r="S44" t="str">
@@ -3148,7 +3148,7 @@
       </c>
     </row>
     <row r="45" xml:space="preserve">
-      <c r="A45">
+      <c r="A45" t="str">
         <v>81628</v>
       </c>
       <c r="B45" t="str">
@@ -3175,7 +3175,7 @@
       <c r="H45" t="str">
         <v>Alexsandro Teixeira Monteiro</v>
       </c>
-      <c r="I45">
+      <c r="I45" t="str">
         <v>150</v>
       </c>
       <c r="J45" t="str">
@@ -3193,7 +3193,7 @@
       <c r="N45" t="str">
         <v>252079</v>
       </c>
-      <c r="O45">
+      <c r="O45" t="str">
         <v>46027.58320601852</v>
       </c>
       <c r="P45" t="str">
@@ -3202,7 +3202,7 @@
       <c r="Q45" t="str">
         <v>34705501829</v>
       </c>
-      <c r="R45">
+      <c r="R45" t="str">
         <v>46027.6141087963</v>
       </c>
       <c r="S45" t="str">
@@ -3213,7 +3213,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46">
+      <c r="A46" t="str">
         <v>81627</v>
       </c>
       <c r="B46" t="str">
@@ -3237,7 +3237,7 @@
       <c r="H46" t="str">
         <v>Carlos Alberto da Silva</v>
       </c>
-      <c r="I46">
+      <c r="I46" t="str">
         <v>2700</v>
       </c>
       <c r="J46" t="str">
@@ -3255,7 +3255,7 @@
       <c r="N46" t="str">
         <v>252076</v>
       </c>
-      <c r="O46">
+      <c r="O46" t="str">
         <v>46027.58148148148</v>
       </c>
       <c r="P46" t="str">
@@ -3264,7 +3264,7 @@
       <c r="Q46" t="str">
         <v>CNPJ 58237197/00001-67</v>
       </c>
-      <c r="R46">
+      <c r="R46" t="str">
         <v>46027.61403935185</v>
       </c>
       <c r="S46" t="str">
@@ -3275,7 +3275,7 @@
       </c>
     </row>
     <row r="47" xml:space="preserve">
-      <c r="A47">
+      <c r="A47" t="str">
         <v>81625</v>
       </c>
       <c r="B47" t="str">
@@ -3300,7 +3300,7 @@
       <c r="G47" t="str">
         <v>Layza Nascimento Fagundes da Costa</v>
       </c>
-      <c r="I47">
+      <c r="I47" t="str">
         <v>500</v>
       </c>
       <c r="J47" t="str">
@@ -3318,7 +3318,7 @@
       <c r="N47" t="str">
         <v>252077</v>
       </c>
-      <c r="O47">
+      <c r="O47" t="str">
         <v>46027.57561342593</v>
       </c>
       <c r="P47" t="str">
@@ -3327,7 +3327,7 @@
       <c r="Q47" t="str">
         <v>CPF 45989904819</v>
       </c>
-      <c r="R47">
+      <c r="R47" t="str">
         <v>46027.61399305556</v>
       </c>
       <c r="S47" t="str">
@@ -3338,7 +3338,7 @@
       </c>
     </row>
     <row r="48" xml:space="preserve">
-      <c r="A48">
+      <c r="A48" t="str">
         <v>81616</v>
       </c>
       <c r="B48" t="str">
@@ -3365,7 +3365,7 @@
       <c r="H48" t="str">
         <v>Orney da Silva</v>
       </c>
-      <c r="I48">
+      <c r="I48" t="str">
         <v>150</v>
       </c>
       <c r="J48" t="str">
@@ -3383,13 +3383,13 @@
       <c r="N48" t="str">
         <v>252025</v>
       </c>
-      <c r="O48">
+      <c r="O48" t="str">
         <v>46027.50078703704</v>
       </c>
       <c r="P48" t="str">
         <v>Faísca auto elétrica</v>
       </c>
-      <c r="R48">
+      <c r="R48" t="str">
         <v>46027.720601851855</v>
       </c>
       <c r="S48" t="str">
@@ -3400,7 +3400,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49">
+      <c r="A49" t="str">
         <v>81608</v>
       </c>
       <c r="B49" t="str">
@@ -3424,7 +3424,7 @@
       <c r="H49" t="str">
         <v>GILVANIA MARIA ARAUJO</v>
       </c>
-      <c r="I49">
+      <c r="I49" t="str">
         <v>40</v>
       </c>
       <c r="J49" t="str">
@@ -3442,7 +3442,7 @@
       <c r="N49" t="str">
         <v>OS-252008</v>
       </c>
-      <c r="O49">
+      <c r="O49" t="str">
         <v>46027.4659837963</v>
       </c>
       <c r="P49" t="str">
@@ -3451,7 +3451,7 @@
       <c r="Q49" t="str">
         <v xml:space="preserve">CNPJ-97.534.937/0001-89 </v>
       </c>
-      <c r="R49">
+      <c r="R49" t="str">
         <v>46027.516921296294</v>
       </c>
       <c r="S49" t="str">
@@ -3462,7 +3462,7 @@
       </c>
     </row>
     <row r="50" xml:space="preserve">
-      <c r="A50">
+      <c r="A50" t="str">
         <v>81605</v>
       </c>
       <c r="B50" t="str">
@@ -3489,7 +3489,7 @@
       <c r="H50" t="str">
         <v>-</v>
       </c>
-      <c r="I50">
+      <c r="I50" t="str">
         <v>400</v>
       </c>
       <c r="J50" t="str">
@@ -3507,7 +3507,7 @@
       <c r="N50" t="str">
         <v>251982</v>
       </c>
-      <c r="O50">
+      <c r="O50" t="str">
         <v>46027.43572916667</v>
       </c>
       <c r="P50" t="str">
@@ -3516,7 +3516,7 @@
       <c r="Q50" t="str">
         <v>CNPJ: 13.176.246/0001-60</v>
       </c>
-      <c r="R50">
+      <c r="R50" t="str">
         <v>46027.482303240744</v>
       </c>
       <c r="S50" t="str">
@@ -3536,7 +3536,7 @@
       </c>
     </row>
     <row r="51" xml:space="preserve">
-      <c r="A51">
+      <c r="A51" t="str">
         <v>81599</v>
       </c>
       <c r="B51" t="str">
@@ -3562,7 +3562,7 @@
       <c r="H51" t="str">
         <v>Leonardo Brandão dos Santos</v>
       </c>
-      <c r="I51">
+      <c r="I51" t="str">
         <v>120</v>
       </c>
       <c r="J51" t="str">
@@ -3580,10 +3580,10 @@
       <c r="N51" t="str">
         <v>251934</v>
       </c>
-      <c r="O51">
+      <c r="O51" t="str">
         <v>46027.4034375</v>
       </c>
-      <c r="R51">
+      <c r="R51" t="str">
         <v>46027.61262731482</v>
       </c>
       <c r="S51" t="str">
@@ -3594,7 +3594,7 @@
       </c>
     </row>
     <row r="52" xml:space="preserve">
-      <c r="A52">
+      <c r="A52" t="str">
         <v>81596</v>
       </c>
       <c r="B52" t="str">
@@ -3623,7 +3623,7 @@
       <c r="H52" t="str">
         <v>-</v>
       </c>
-      <c r="I52">
+      <c r="I52" t="str">
         <v>63.8</v>
       </c>
       <c r="J52" t="str">
@@ -3641,7 +3641,7 @@
       <c r="N52" t="str">
         <v>248088</v>
       </c>
-      <c r="O52">
+      <c r="O52" t="str">
         <v>46027.39142361111</v>
       </c>
       <c r="P52" t="str">
@@ -3650,7 +3650,7 @@
       <c r="Q52" t="str">
         <v>CNPJ:05.212.047/0001-32</v>
       </c>
-      <c r="R52">
+      <c r="R52" t="str">
         <v>46027.481875</v>
       </c>
       <c r="S52" t="str">
@@ -3670,7 +3670,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53">
+      <c r="A53" t="str">
         <v>81594</v>
       </c>
       <c r="B53" t="str">
@@ -3694,7 +3694,7 @@
       <c r="H53" t="str">
         <v xml:space="preserve">JOSE CLAUDIO RODRIGUES DE OLIVEIRA </v>
       </c>
-      <c r="I53">
+      <c r="I53" t="str">
         <v>130</v>
       </c>
       <c r="J53" t="str">
@@ -3712,7 +3712,7 @@
       <c r="N53" t="str">
         <v>OS-251900</v>
       </c>
-      <c r="O53">
+      <c r="O53" t="str">
         <v>46027.38064814815</v>
       </c>
       <c r="P53" t="str">
@@ -3721,7 +3721,7 @@
       <c r="Q53" t="str">
         <v>CPF-050.719.475-60</v>
       </c>
-      <c r="R53">
+      <c r="R53" t="str">
         <v>46027.40923611111</v>
       </c>
       <c r="S53" t="str">
@@ -3732,7 +3732,7 @@
       </c>
     </row>
     <row r="54" xml:space="preserve">
-      <c r="A54">
+      <c r="A54" t="str">
         <v>81591</v>
       </c>
       <c r="B54" t="str">
@@ -3757,7 +3757,7 @@
       <c r="H54" t="str">
         <v>Luciano Babuia</v>
       </c>
-      <c r="I54">
+      <c r="I54" t="str">
         <v>500</v>
       </c>
       <c r="J54" t="str">
@@ -3775,7 +3775,7 @@
       <c r="N54" t="str">
         <v>251883</v>
       </c>
-      <c r="O54">
+      <c r="O54" t="str">
         <v>46027.3590625</v>
       </c>
       <c r="P54" t="str">
@@ -3784,7 +3784,7 @@
       <c r="Q54" t="str">
         <v>40277899893</v>
       </c>
-      <c r="R54">
+      <c r="R54" t="str">
         <v>46027.4090162037</v>
       </c>
       <c r="S54" t="str">
@@ -3795,7 +3795,7 @@
       </c>
     </row>
     <row r="55" xml:space="preserve">
-      <c r="A55">
+      <c r="A55" t="str">
         <v>81570</v>
       </c>
       <c r="B55" t="str">
@@ -3821,7 +3821,7 @@
       <c r="H55" t="str">
         <v>NÃO POSSUI</v>
       </c>
-      <c r="I55">
+      <c r="I55" t="str">
         <v>500</v>
       </c>
       <c r="J55" t="str">
@@ -3839,13 +3839,13 @@
       <c r="N55" t="str">
         <v>251851</v>
       </c>
-      <c r="O55">
+      <c r="O55" t="str">
         <v>46025.58579861111</v>
       </c>
       <c r="P55" t="str">
         <v>JULIO CESAR DA SILVA</v>
       </c>
-      <c r="R55">
+      <c r="R55" t="str">
         <v>46025.63108796296</v>
       </c>
       <c r="S55" t="str">
@@ -3856,7 +3856,7 @@
       </c>
     </row>
     <row r="56" xml:space="preserve">
-      <c r="A56">
+      <c r="A56" t="str">
         <v>81565</v>
       </c>
       <c r="B56" t="str">
@@ -3882,7 +3882,7 @@
       <c r="H56" t="str">
         <v>RENILDO CAMPOS NOGUE</v>
       </c>
-      <c r="I56">
+      <c r="I56" t="str">
         <v>60</v>
       </c>
       <c r="J56" t="str">
@@ -3900,10 +3900,10 @@
       <c r="N56" t="str">
         <v>251847</v>
       </c>
-      <c r="O56">
+      <c r="O56" t="str">
         <v>46025.57491898148</v>
       </c>
-      <c r="R56">
+      <c r="R56" t="str">
         <v>46025.630960648145</v>
       </c>
       <c r="S56" t="str">
@@ -3914,7 +3914,7 @@
       </c>
     </row>
     <row r="57" xml:space="preserve">
-      <c r="A57">
+      <c r="A57" t="str">
         <v>81543</v>
       </c>
       <c r="B57" t="str">
@@ -3940,7 +3940,7 @@
       <c r="H57" t="str">
         <v>LUCIENE BATISTA DA SILVA</v>
       </c>
-      <c r="I57">
+      <c r="I57" t="str">
         <v>3100</v>
       </c>
       <c r="J57" t="str">
@@ -3958,13 +3958,13 @@
       <c r="N57" t="str">
         <v>251830</v>
       </c>
-      <c r="O57">
+      <c r="O57" t="str">
         <v>46025.415127314816</v>
       </c>
       <c r="P57" t="str">
         <v>Msg salvador Comércio de baterias Fox BATERIAS</v>
       </c>
-      <c r="R57">
+      <c r="R57" t="str">
         <v>46025.44116898148</v>
       </c>
       <c r="S57" t="str">
@@ -3975,7 +3975,7 @@
       </c>
     </row>
     <row r="58" xml:space="preserve">
-      <c r="A58">
+      <c r="A58" t="str">
         <v>81538</v>
       </c>
       <c r="B58" t="str">
@@ -4001,7 +4001,7 @@
       <c r="G58" t="str">
         <v>Layza Nascimento Fagundes da Costa</v>
       </c>
-      <c r="I58">
+      <c r="I58" t="str">
         <v>410</v>
       </c>
       <c r="J58" t="str">
@@ -4019,7 +4019,7 @@
       <c r="N58" t="str">
         <v xml:space="preserve">251822  - 251827 </v>
       </c>
-      <c r="O58">
+      <c r="O58" t="str">
         <v>46025.39221064815</v>
       </c>
       <c r="P58" t="str">
@@ -4028,7 +4028,7 @@
       <c r="Q58" t="str">
         <v>50497778000126</v>
       </c>
-      <c r="R58">
+      <c r="R58" t="str">
         <v>46025.42534722222</v>
       </c>
       <c r="S58" t="str">
@@ -4036,7 +4036,7 @@
       </c>
     </row>
     <row r="59" xml:space="preserve">
-      <c r="A59">
+      <c r="A59" t="str">
         <v>81534</v>
       </c>
       <c r="B59" t="str">
@@ -4062,7 +4062,7 @@
       <c r="H59" t="str">
         <v>WESLEI DOS SANTOS PONTES</v>
       </c>
-      <c r="I59">
+      <c r="I59" t="str">
         <v>350</v>
       </c>
       <c r="J59" t="str">
@@ -4080,13 +4080,13 @@
       <c r="N59" t="str">
         <v>251796</v>
       </c>
-      <c r="O59">
+      <c r="O59" t="str">
         <v>46025.30756944444</v>
       </c>
       <c r="P59" t="str">
         <v xml:space="preserve">DAVID FRANCISCO </v>
       </c>
-      <c r="R59">
+      <c r="R59" t="str">
         <v>46025.440983796296</v>
       </c>
       <c r="S59" t="str">
@@ -4097,7 +4097,7 @@
       </c>
     </row>
     <row r="60" xml:space="preserve">
-      <c r="A60">
+      <c r="A60" t="str">
         <v>81525</v>
       </c>
       <c r="B60" t="str">
@@ -4124,7 +4124,7 @@
       <c r="H60" t="str">
         <v xml:space="preserve">Átila Pereira de Sousa </v>
       </c>
-      <c r="I60">
+      <c r="I60" t="str">
         <v>1090</v>
       </c>
       <c r="J60" t="str">
@@ -4142,13 +4142,13 @@
       <c r="N60" t="str">
         <v>251740</v>
       </c>
-      <c r="O60">
+      <c r="O60" t="str">
         <v>46024.690567129626</v>
       </c>
       <c r="P60" t="str">
         <v xml:space="preserve">Alex Sousa </v>
       </c>
-      <c r="R60">
+      <c r="R60" t="str">
         <v>46025.4249537037</v>
       </c>
       <c r="S60" t="str">
@@ -4159,7 +4159,7 @@
       </c>
     </row>
     <row r="61" xml:space="preserve">
-      <c r="A61">
+      <c r="A61" t="str">
         <v>81520</v>
       </c>
       <c r="B61" t="str">
@@ -4192,7 +4192,7 @@
       <c r="H61" t="str">
         <v>-</v>
       </c>
-      <c r="I61">
+      <c r="I61" t="str">
         <v>750</v>
       </c>
       <c r="J61" t="str">
@@ -4210,7 +4210,7 @@
       <c r="N61" t="str">
         <v>O.S: 251713</v>
       </c>
-      <c r="O61">
+      <c r="O61" t="str">
         <v>46024.65493055555</v>
       </c>
       <c r="P61" t="str">
@@ -4219,7 +4219,7 @@
       <c r="Q61" t="str">
         <v>CPF 02175621405</v>
       </c>
-      <c r="R61">
+      <c r="R61" t="str">
         <v>46024.67921296296</v>
       </c>
       <c r="S61" t="str">
@@ -4239,7 +4239,7 @@
       </c>
     </row>
     <row r="62" xml:space="preserve">
-      <c r="A62">
+      <c r="A62" t="str">
         <v>81507</v>
       </c>
       <c r="B62" t="str">
@@ -4266,7 +4266,7 @@
       <c r="H62" t="str">
         <v>Kauê aparecido de Campos Tavares da Silva</v>
       </c>
-      <c r="I62">
+      <c r="I62" t="str">
         <v>80</v>
       </c>
       <c r="J62" t="str">
@@ -4284,13 +4284,13 @@
       <c r="N62" t="str">
         <v xml:space="preserve">251680 </v>
       </c>
-      <c r="O62">
+      <c r="O62" t="str">
         <v>46024.595347222225</v>
       </c>
       <c r="P62" t="str">
         <v>Kauê aparecido de Campos Tavares da Silva</v>
       </c>
-      <c r="R62">
+      <c r="R62" t="str">
         <v>46024.65561342592</v>
       </c>
       <c r="S62" t="str">
@@ -4301,7 +4301,7 @@
       </c>
     </row>
     <row r="63" xml:space="preserve">
-      <c r="A63">
+      <c r="A63" t="str">
         <v>81499</v>
       </c>
       <c r="B63" t="str">
@@ -4327,7 +4327,7 @@
       <c r="H63" t="str">
         <v>NÃO POSSUI</v>
       </c>
-      <c r="I63">
+      <c r="I63" t="str">
         <v>150</v>
       </c>
       <c r="J63" t="str">
@@ -4345,13 +4345,13 @@
       <c r="N63" t="str">
         <v>251638</v>
       </c>
-      <c r="O63">
+      <c r="O63" t="str">
         <v>46024.54311342593</v>
       </c>
       <c r="P63" t="str">
         <v>Borracharia Bom Jesus</v>
       </c>
-      <c r="R63">
+      <c r="R63" t="str">
         <v>46024.67290509259</v>
       </c>
       <c r="S63" t="str">
@@ -4362,7 +4362,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64">
+      <c r="A64" t="str">
         <v>81491</v>
       </c>
       <c r="B64" t="str">
@@ -4386,7 +4386,7 @@
       <c r="H64" t="str">
         <v>Eduardo Henrique Aguiar de Paiva</v>
       </c>
-      <c r="I64">
+      <c r="I64" t="str">
         <v>200</v>
       </c>
       <c r="J64" t="str">
@@ -4404,13 +4404,13 @@
       <c r="N64" t="str">
         <v>251609</v>
       </c>
-      <c r="O64">
+      <c r="O64" t="str">
         <v>46024.502592592595</v>
       </c>
       <c r="P64" t="str">
         <v>Eduardo Henrique Aguiar de Paiva</v>
       </c>
-      <c r="R64">
+      <c r="R64" t="str">
         <v>46024.598703703705</v>
       </c>
       <c r="S64" t="str">
@@ -4421,7 +4421,7 @@
       </c>
     </row>
     <row r="65" xml:space="preserve">
-      <c r="A65">
+      <c r="A65" t="str">
         <v>81489</v>
       </c>
       <c r="B65" t="str">
@@ -4446,7 +4446,7 @@
       <c r="H65" t="str">
         <v xml:space="preserve">Francisco Carlos da Silva Cruz </v>
       </c>
-      <c r="I65">
+      <c r="I65" t="str">
         <v>70</v>
       </c>
       <c r="J65" t="str">
@@ -4464,13 +4464,13 @@
       <c r="N65" t="str">
         <v>251600</v>
       </c>
-      <c r="O65">
+      <c r="O65" t="str">
         <v>46024.487708333334</v>
       </c>
       <c r="P65" t="str">
         <v xml:space="preserve">Francisco Carlos da Silva Cruz </v>
       </c>
-      <c r="R65">
+      <c r="R65" t="str">
         <v>46024.519375</v>
       </c>
       <c r="S65" t="str">
@@ -4481,7 +4481,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66">
+      <c r="A66" t="str">
         <v>81487</v>
       </c>
       <c r="B66" t="str">
@@ -4505,7 +4505,7 @@
       <c r="H66" t="str">
         <v>JANDSON SANTANA DE OLIVEIRA</v>
       </c>
-      <c r="I66">
+      <c r="I66" t="str">
         <v>100</v>
       </c>
       <c r="J66" t="str">
@@ -4523,13 +4523,13 @@
       <c r="N66" t="str">
         <v>251586</v>
       </c>
-      <c r="O66">
+      <c r="O66" t="str">
         <v>46024.47454861111</v>
       </c>
       <c r="P66" t="str">
         <v>JANDSON SANTANA DE OLIVEIRA</v>
       </c>
-      <c r="R66">
+      <c r="R66" t="str">
         <v>46024.51939814815</v>
       </c>
       <c r="S66" t="str">
@@ -4540,7 +4540,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67">
+      <c r="A67" t="str">
         <v>81486</v>
       </c>
       <c r="B67" t="str">
@@ -4564,7 +4564,7 @@
       <c r="H67" t="str">
         <v>Bruno ricardo de brito</v>
       </c>
-      <c r="I67">
+      <c r="I67" t="str">
         <v>55</v>
       </c>
       <c r="J67" t="str">
@@ -4582,13 +4582,13 @@
       <c r="N67" t="str">
         <v xml:space="preserve"> UBC4G81</v>
       </c>
-      <c r="O67">
+      <c r="O67" t="str">
         <v>46024.46501157407</v>
       </c>
       <c r="P67" t="str">
         <v>Bruno ricardo de brito</v>
       </c>
-      <c r="R67">
+      <c r="R67" t="str">
         <v>46024.51931712963</v>
       </c>
       <c r="S67" t="str">
@@ -4599,7 +4599,7 @@
       </c>
     </row>
     <row r="68" xml:space="preserve">
-      <c r="A68">
+      <c r="A68" t="str">
         <v>81479</v>
       </c>
       <c r="B68" t="str">
@@ -4625,7 +4625,7 @@
       <c r="H68" t="str">
         <v>IRAM MOREIRA DOS SANTOS</v>
       </c>
-      <c r="I68">
+      <c r="I68" t="str">
         <v>640</v>
       </c>
       <c r="J68" t="str">
@@ -4643,13 +4643,13 @@
       <c r="N68" t="str">
         <v>251555</v>
       </c>
-      <c r="O68">
+      <c r="O68" t="str">
         <v>46024.42199074074</v>
       </c>
       <c r="P68" t="str">
         <v>BRUNO BELOTO PIZOL</v>
       </c>
-      <c r="R68">
+      <c r="R68" t="str">
         <v>46024.51929398148</v>
       </c>
       <c r="S68" t="str">

</xml_diff>